<commit_message>
Schema 0.1.3: station field (reach-filtered) + PARENT_MISMATCH QA check
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BLDQF1jq1tUN6A8Y3GgMFD
</commit_message>
<xml_diff>
--- a/form/whatcom_salmon.xlsx
+++ b/form/whatcom_salmon.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O17"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -480,20 +480,25 @@
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
+          <t>choice_filter</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
           <t>appearance</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>bind::esri:fieldType</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>bind::esri:fieldLength</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>body::accuracyThreshold</t>
         </is>
@@ -523,6 +528,7 @@
       <c r="M2" t="inlineStr"/>
       <c r="N2" t="inlineStr"/>
       <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -568,6 +574,7 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -615,10 +622,11 @@
       </c>
       <c r="L4" t="inlineStr"/>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="n">
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="n">
         <v>50</v>
       </c>
-      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -656,21 +664,22 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr"/>
       <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>geopoint</t>
+          <t>select_one station</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>location</t>
+          <t>station</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Observation location</t>
+          <t>Station</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -681,7 +690,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Observation location is required</t>
+          <t>Station is required</t>
         </is>
       </c>
       <c r="G6" t="inlineStr"/>
@@ -689,101 +698,108 @@
       <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr"/>
       <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>reach=${reach}</t>
+        </is>
+      </c>
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr"/>
-      <c r="O6" t="n">
-        <v>50</v>
-      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>hidden</t>
+          <t>geopoint</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>gps_accuracy_m</t>
+          <t>location</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>GPS horizontal accuracy (m)</t>
+          <t>Observation location</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
-      <c r="F7" t="inlineStr"/>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Observation location is required</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>pulldata("@geopoint", ${location}, "horizontalAccuracy")</t>
-        </is>
-      </c>
+      <c r="K7" t="inlineStr"/>
       <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr">
-        <is>
-          <t>esriFieldTypeDouble</t>
-        </is>
-      </c>
+      <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr"/>
       <c r="O7" t="inlineStr"/>
+      <c r="P7" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>select_one obs_type</t>
+          <t>hidden</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>obs_type</t>
+          <t>gps_accuracy_m</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Observation type</t>
+          <t>GPS horizontal accuracy (m)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Observation type is required</t>
-        </is>
-      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>pulldata("@geopoint", ${location}, "horizontalAccuracy")</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr"/>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>esriFieldTypeDouble</t>
+        </is>
+      </c>
       <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>select_one species</t>
+          <t>select_one obs_type</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>species</t>
+          <t>obs_type</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Species</t>
+          <t>Observation type</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -794,37 +810,34 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Species is required for this observation type</t>
+          <t>Observation type is required</t>
         </is>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>${obs_type} = 'live_fish' or ${obs_type} = 'carcass' or ${obs_type} = 'redd'</t>
-        </is>
-      </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr"/>
       <c r="K9" t="inlineStr"/>
       <c r="L9" t="inlineStr"/>
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr"/>
       <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>integer</t>
+          <t>select_one species</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>count</t>
+          <t>species</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Count</t>
+          <t>Species</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -835,22 +848,14 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Count is required for this observation type</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>. &gt;= 0 and . &lt;= 500</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Must be 0-500</t>
-        </is>
-      </c>
+          <t>Species is required for this observation type</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>${obs_type} = 'live_fish' or ${obs_type} = 'carcass'</t>
+          <t>${obs_type} = 'live_fish' or ${obs_type} = 'carcass' or ${obs_type} = 'redd'</t>
         </is>
       </c>
       <c r="J10" t="inlineStr"/>
@@ -859,6 +864,7 @@
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr"/>
       <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -868,12 +874,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>redd_count</t>
+          <t>count</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Redd count</t>
+          <t>Count</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -884,22 +890,22 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Redd count is required for this observation type</t>
+          <t>Count is required for this observation type</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>. &gt;= 0 and . &lt;= 100</t>
+          <t>. &gt;= 0 and . &lt;= 500</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Must be 0-100</t>
+          <t>Must be 0-500</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>${obs_type} = 'redd'</t>
+          <t>${obs_type} = 'live_fish' or ${obs_type} = 'carcass'</t>
         </is>
       </c>
       <c r="J11" t="inlineStr"/>
@@ -908,21 +914,22 @@
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr"/>
       <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>select_one water_clarity</t>
+          <t>integer</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>water_clarity</t>
+          <t>redd_count</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Water clarity</t>
+          <t>Redd count</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -933,33 +940,46 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Water clarity is required</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
+          <t>Redd count is required for this observation type</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>. &gt;= 0 and . &lt;= 100</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Must be 0-100</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>${obs_type} = 'redd'</t>
+        </is>
+      </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
       <c r="L12" t="inlineStr"/>
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr"/>
       <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>select_one flow</t>
+          <t>select_one water_clarity</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>flow</t>
+          <t>water_clarity</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Flow</t>
+          <t>Water clarity</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -970,7 +990,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Flow is required</t>
+          <t>Water clarity is required</t>
         </is>
       </c>
       <c r="G13" t="inlineStr"/>
@@ -982,26 +1002,35 @@
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>select_one weather</t>
+          <t>select_one flow</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>weather</t>
+          <t>flow</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Weather</t>
+          <t>Flow</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
-      <c r="F14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Flow is required</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
@@ -1011,21 +1040,22 @@
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>select_one weather</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>photo</t>
+          <t>weather</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Photo</t>
+          <t>Weather</t>
         </is>
       </c>
       <c r="D15" t="inlineStr"/>
@@ -1040,84 +1070,117 @@
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>notes</t>
+          <t>photo</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Notes</t>
+          <t>Photo</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>string-length(.) &lt;= 250</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>Max 250 characters</t>
-        </is>
-      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="L16" t="inlineStr"/>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="n">
-        <v>250</v>
-      </c>
+      <c r="N16" t="inlineStr"/>
       <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>hidden</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>qa_flag</t>
+          <t>notes</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>QA flag</t>
+          <t>Notes</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>string-length(.) &lt;= 250</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Max 250 characters</t>
+        </is>
+      </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
       <c r="L17" t="inlineStr"/>
       <c r="M17" t="inlineStr">
         <is>
+          <t>multiline</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr"/>
+      <c r="O17" t="n">
+        <v>250</v>
+      </c>
+      <c r="P17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>hidden</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>qa_flag</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>QA flag</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr"/>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr"/>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
           <t>esriFieldTypeString</t>
         </is>
       </c>
-      <c r="N17" t="n">
+      <c r="O18" t="n">
         <v>255</v>
       </c>
-      <c r="O17" t="inlineStr"/>
+      <c r="P18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1130,7 +1193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1149,6 +1212,11 @@
           <t>label</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>reach</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1166,6 +1234,7 @@
           <t>R1: Mouth to Maritime Heritage Park</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1183,6 +1252,7 @@
           <t>R2: Maritime Heritage Park to Woburn St</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1200,6 +1270,7 @@
           <t>R3: Woburn St to WWU Fisheries Rental</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1217,363 +1288,495 @@
           <t>R4: WWU Rental to Lake Outlet</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>obs_type</t>
+          <t>station</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>live_fish</t>
+          <t>R1-S1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Live fish</t>
+          <t>R1-S1: Holly St bridge</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>R1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>obs_type</t>
+          <t>station</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>carcass</t>
+          <t>R2-S1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Carcass</t>
+          <t>R2-S1: Meador bridge</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>R2</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>obs_type</t>
+          <t>station</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>redd</t>
+          <t>R2-S2</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Redd</t>
+          <t>R2-S2: Woburn St bridge</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>R2</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>obs_type</t>
+          <t>station</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>habitat</t>
+          <t>R3-S1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Habitat feature</t>
+          <t>R3-S1: Whatcom Falls Park</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>R3</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>obs_type</t>
+          <t>station</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>no_fish</t>
+          <t>R4-S1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>No fish seen</t>
+          <t>R4-S1: Electric Ave bridge</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>R4</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>species</t>
+          <t>obs_type</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>chum</t>
+          <t>live_fish</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Chum</t>
-        </is>
-      </c>
+          <t>Live fish</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>species</t>
+          <t>obs_type</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>coho</t>
+          <t>carcass</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Coho</t>
-        </is>
-      </c>
+          <t>Carcass</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>species</t>
+          <t>obs_type</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>chinook</t>
+          <t>redd</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Chinook</t>
-        </is>
-      </c>
+          <t>Redd</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>species</t>
+          <t>obs_type</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>pink</t>
+          <t>habitat</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pink</t>
-        </is>
-      </c>
+          <t>Habitat feature</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>species</t>
+          <t>obs_type</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>unk_salmonid</t>
+          <t>no_fish</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Unknown salmonid</t>
-        </is>
-      </c>
+          <t>No fish seen</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>water_clarity</t>
+          <t>species</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>clear</t>
+          <t>chum</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Clear</t>
-        </is>
-      </c>
+          <t>Chum</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>water_clarity</t>
+          <t>species</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>slight_turbid</t>
+          <t>coho</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Slightly turbid</t>
-        </is>
-      </c>
+          <t>Coho</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>water_clarity</t>
+          <t>species</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>turbid</t>
+          <t>chinook</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Turbid</t>
-        </is>
-      </c>
+          <t>Chinook</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>flow</t>
+          <t>species</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>pink</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Low</t>
-        </is>
-      </c>
+          <t>Pink</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>flow</t>
+          <t>species</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>normal</t>
+          <t>unk_salmonid</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Normal</t>
-        </is>
-      </c>
+          <t>Unknown salmonid</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>flow</t>
+          <t>water_clarity</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>clear</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>High</t>
-        </is>
-      </c>
+          <t>Clear</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>weather</t>
+          <t>water_clarity</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>clear</t>
+          <t>slight_turbid</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Clear</t>
-        </is>
-      </c>
+          <t>Slightly turbid</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>weather</t>
+          <t>water_clarity</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>overcast</t>
+          <t>turbid</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Overcast</t>
-        </is>
-      </c>
+          <t>Turbid</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>weather</t>
+          <t>flow</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>light_rain</t>
+          <t>low</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Light rain</t>
-        </is>
-      </c>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>weather</t>
+          <t>flow</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>heavy_rain</t>
+          <t>normal</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Heavy rain</t>
-        </is>
-      </c>
+          <t>Normal</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>flow</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>weather</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>clear</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Clear</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>overcast</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Overcast</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>light_rain</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Light rain</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>heavy_rain</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Heavy rain</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>weather</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
         <is>
           <t>fog</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>Fog</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1624,12 +1827,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026100221</t>
+          <t>2026100610</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>concat(${reach}, ' - ', ${obs_type})</t>
+          <t>concat(${station}, ' - ', ${obs_type})</t>
         </is>
       </c>
     </row>

</xml_diff>